<commit_message>
fix: align paper text and output columns with F-test-first logic
- Fix §3 paper text to describe F-test as primary criterion (not engineering thresholds)
- Fix §8 to say "F检验为统计依据" instead of "同时考虑统计显著性和工程效应量"
- Fix estimates_summary column "是否采用系统偏差修正" to report actual decision
- Add "工程效应量达标" as separate reference column
- Fix result.xlsx template detection to scan all columns for "注意"/"填写范例"
- Restore clean template from 附件4.xlsx
- Regenerate all binary outputs with correct Problem 3 bias values
</commit_message>
<xml_diff>
--- a/2026_B题/outputs/estimates_summary.xlsx
+++ b/2026_B题/outputs/estimates_summary.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,96 +425,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>问题</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>方式1时间偏差_s</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>方式2相对方式1时间偏差_delta_s</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>delta_95%CI_lower_s</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>delta_95%CI_upper_s</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>采用的系统偏差_x_m</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>采用的系统偏差_y_m</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>候选系统偏差_x_m</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>候选系统偏差_y_m</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>是否统计显著</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>是否采用系统偏差修正</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>工程效应量达标</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>F统计量</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>F检验p值</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>重叠时长_s</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>重叠样本数</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>带偏差模型MSE</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>无偏差模型MSE</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>误差下降比例</t>
         </is>
@@ -542,17 +559,22 @@
           <t>否</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="n">
         <v>700.3500010957835</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>7004</v>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -588,25 +610,30 @@
           <t>是</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>195086.9059078202</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>690.0020947843262</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>6900</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.2689992178130305</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>15.48448924239056</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>0.9826278275245518</v>
       </c>
     </row>
@@ -618,19 +645,19 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>-367.9164073195533</v>
+        <v>-367.9213835976812</v>
       </c>
       <c r="D4" t="n">
-        <v>-367.9237106191135</v>
+        <v>-367.9281963250401</v>
       </c>
       <c r="E4" t="n">
-        <v>-367.9085541483682</v>
+        <v>-367.9133494967213</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>-0.1494990834440912</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>-0.2095227637940198</v>
       </c>
       <c r="H4" t="n">
         <v>-0.1494990834440912</v>
@@ -645,28 +672,33 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>否</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>25.17272149771372</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>1.440136898622768e-11</v>
       </c>
-      <c r="N4" t="n">
-        <v>299.9964073195533</v>
-      </c>
       <c r="O4" t="n">
+        <v>300.0013835976812</v>
+      </c>
+      <c r="P4" t="n">
         <v>3000</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>3.748272589657936</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>3.811217367507818</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>0.01651566199989328</v>
       </c>
     </row>

</xml_diff>